<commit_message>
List TODO v každém sezónním sešitu + read-only analytické nástroje
Zachován formát 1 sešit = 1 sezóna (kvůli ruční kontrole kolegou).

- Do všech 65 sešitů přidán list 'TODO' jen s položkami té sezóny
  (bold hlavička, autofiltr, zmrazený řádek, sloupce pro kolegu);
  paralelní [TBD] řádky v NOTES dle konvence D19. Idempotentní
  (re-run nepřidává duplikáty). Datové listy beze změny.
- apply_todo_sheets.py — znovuspustitelná distribuce TODO_continuity.md
- build_db.py / health.py — VOLITELNÉ read-only nástroje (konsolidovaná
  SQLite + report zdraví DB); negenerují nic do sešitů, artefakty
  gitignorovány. HEALTH.md = snapshot stavu.

https://claude.ai/code/session_01KztM35VfsFKiyd6BJa25sx
</commit_message>
<xml_diff>
--- a/data/S1951_52_FINAL.xlsx
+++ b/data/S1951_52_FINAL.xlsx
@@ -34,8 +34,11 @@
     <sheet name="SERIES" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="CLUBS" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="META" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="TODO" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="27" hidden="1">'TODO'!$A$1:$F$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -43,7 +46,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +61,12 @@
       <name val="Arial"/>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -81,6 +88,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00305496"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -94,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -104,6 +116,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -18541,7 +18559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18949,6 +18967,47 @@
       <c r="D18" t="inlineStr">
         <is>
           <t>T</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>[TBD] prev_club_id: CLUB_S1951_52_0131 'Sokol Senec' ROZBITÝ prev CLUB_S1949_50_0472 (neexist.), bez jednoznačného kandidáta — ponecháno</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TODO-auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>[TBD] fate: CLUB_S1951_52_0400 fate nekonzist. ['sestup', 'setrval'] → 'sestup' (cross-ref=ne) — ověřit</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>TODO-auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>NODE_S1951_52_0009</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>[TBD] pyramida: SYSTEM NODE_S1951_52_0009 'Mistrovství Slovenska' (L15, parent=NODE_S1951_52_0006) vnořená baráž — feeds_into ponecháno prázdné (ověřit cíl ručně)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>TODO-auto</t>
         </is>
       </c>
     </row>
@@ -21535,8 +21594,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -21604,7 +21661,6 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
@@ -43286,6 +43342,127 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>typ</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>popis</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>vyřešeno? (ANO/ne)</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>poznámka kolegy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>prev_club_id</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CLUB_S1951_52_0131</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>CLUB_S1951_52_0131 'Sokol Senec' ROZBITÝ prev CLUB_S1949_50_0472 (neexist.), bez jednoznačného kandidáta — ponecháno</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>fate</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CLUB_S1951_52_0400</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>CLUB_S1951_52_0400 fate nekonzist. ['sestup', 'setrval'] → 'sestup' (cross-ref=ne) — ověřit</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pyramida</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>NODE_S1951_52_0009</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>SYSTEM NODE_S1951_52_0009 'Mistrovství Slovenska' (L15, parent=NODE_S1951_52_0006) vnořená baráž — feeds_into ponecháno prázdné (ověřit cíl ručně)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Křížová kontrola nejvyšší soutěže proti PDF (pořadí pravdy PDF>xlsx): 26 oprav
verify_vs_pdf.py porovnal 10_liga všech 73 sezón se sources/CZE1/*.pdf.
Join přes (GP,GF,GA) + 2. průchod přes ověřené V/R/P. Opraveno z PDF:
- 4× V/R/P (1960/61 Sp. Plzeň, Slavoj ČB; 1963/64 Slovan; 1988/89 Slovan)
- 2× PTS (1963/64 Slovan 30→29, Sp. Plzeň 23→17)
- 20× drobné překlepy GF:GA (ZKL Brno 139→140:41, ATK 80:12→80:13, …)

Po opravách: éra 2-1-0 V+R+P≠GP=0, PTS≠2V+R=3 (jen přenos bodů 1988/89).
4 řádky ponechány k ověření (V/R/P i skóre se rozcházejí — chaotická éra <1965).
Pozn.: wiki je v prostředí blokovaná (WebFetch 403), cross-check běží proti PDF.
README + MASTER_REPORT aktualizovány.
</commit_message>
<xml_diff>
--- a/data/S1951_52_FINAL.xlsx
+++ b/data/S1951_52_FINAL.xlsx
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="M17" t="n">
         <v>4</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="M19" t="n">
         <v>18</v>
@@ -2224,7 +2224,7 @@
         <v>7</v>
       </c>
       <c r="J23" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
1951/52: opravit mistra dle PDF+web (M: České Budějovice → Vítkovice)
PDF Finále mistrovství ČSR: 1. ZSJ Vítkovické železárny KG (8 b, lepší skóre než
ATK Praha 8 b) = mistr. Ověřeno webem (první titul Vítkovic). M badge byl chybně
u SKP České Budějovice, který se do finále vůbec nedostal (3. v základní skupině).
M přesunut na Vítkovice ve finálovém bloku (terminální fáze). META mistr=Vítkovice.
</commit_message>
<xml_diff>
--- a/data/S1951_52_FINAL.xlsx
+++ b/data/S1951_52_FINAL.xlsx
@@ -957,11 +957,6 @@
           <t>SKP České Budějovice</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
       <c r="F7" t="n">
         <v>10</v>
       </c>
@@ -2411,6 +2406,11 @@
       <c r="D26" t="inlineStr">
         <is>
           <t>Vítkovické Železárny</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -18559,7 +18559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -19159,6 +19159,13 @@
       <c r="D34" t="inlineStr">
         <is>
           <t>TODO-auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Mistrovství republiky 1951/52: 3 skupiny po 6 → Finále mistrovství ČSR (2 nejlepší z každé skupiny). Mistr Vítkovice (před ATK Praha na skóre). Doloženo PDF i webem.</t>
         </is>
       </c>
     </row>
@@ -19462,8 +19469,6 @@
           <t>NODE_S1951_52_0001</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -19769,8 +19774,6 @@
           <t>NODE_S1951_52_0009</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>home-away</t>
@@ -19878,8 +19881,6 @@
           <t>NODE_S1951_52_0009</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>home-away</t>
@@ -20249,8 +20250,6 @@
           <t>NODE_S1951_52_0015</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -21139,8 +21138,6 @@
           <t>NODE_S1951_52_0038</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -21800,8 +21797,6 @@
         </is>
       </c>
     </row>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
@@ -21820,8 +21815,6 @@
           <t>Mistrovství republiky (3 sk. × 6 + finále)</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
           <t>vítězové SF</t>
@@ -21894,7 +21887,6 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
@@ -43114,7 +43106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43281,7 +43273,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Reorganizace pyramidy. Oblastní soutěže zrušeny. Liga 18 týmů ve 3 skupinách. Křídla vlasti Olomouc direktivně.</t>
+          <t>Mistr ZSJ Vítkovické železárny KG — vítěz Finále mistrovství ČSR (1., 8 b, lepší skóre než ATK Praha). Vůbec první titul Vítkovic. M badge opraven (byl chybně u SKP České Budějovice, který se do finále nedostal). Struktura: 3 základní skupiny po 6 → finále 6 (po 2 z každé skupiny).</t>
         </is>
       </c>
     </row>
@@ -43582,6 +43574,18 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>Žilinský</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>mistr</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Vítkovické Železárny</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
1951/52 KVAL: opravit skupiny A/B dle DS PDF (Hostivař, Tábor ad.) + poznámky
Ověření kvalifikace o Mistrovství republiky proti DS PDF: interní konzistence
neodhalila rozdíly (data byla balancovaná, ale neúplná). Opraveno dle PDF
(Skupina I: Hostivař 6-5-0-1 47:24, Tábor 5-2-0-3 39:39; Skupina II dle PDF).
Poznámky: slovenský vítěz (Dukla Prešov) nepostoupil — místo něj zařazen nový
armádní tým Křídla vlasti Olomouc (původ jeho 1952/53). Krajské 20* = ruční review.
</commit_message>
<xml_diff>
--- a/data/S1951_52_FINAL.xlsx
+++ b/data/S1951_52_FINAL.xlsx
@@ -16066,10 +16066,10 @@
         </is>
       </c>
       <c r="F5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" t="n">
         <v>5</v>
-      </c>
-      <c r="G5" t="n">
-        <v>4</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -16078,7 +16078,7 @@
         <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -16086,10 +16086,10 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="M5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -16212,7 +16212,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -16221,10 +16221,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -16232,7 +16232,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="M7" t="n">
         <v>4</v>
@@ -18559,7 +18559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -19166,6 +19166,34 @@
       <c r="A35" t="inlineStr">
         <is>
           <t>Mistrovství republiky 1951/52: 3 skupiny po 6 → Finále mistrovství ČSR (2 nejlepší z každé skupiny). Mistr Vítkovice (před ATK Praha na skóre). Doloženo PDF i webem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Kvalifikace o Mistrovství republiky 1951/52 (turnaje krajských přeborníků): Skupina I (Holoubkov), Skupina II (OKD Ostrava), Skupina III = Mistrovství Slovenska (Dukla Prešov).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Vítěz slovenské skupiny (Dukla Prešov) nakonec do Mistrovství republiky NEpostoupil — místo něj byl po svém vzniku rovnou zařazen nový armádní tým Křídla vlasti Olomouc (odtud jeho původ v 1952/53 bez civilního předchůdce).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Kvalifikace o Mistrovství republiky byla nakonec zbytečná: rozhodnuto, že nikdo nesestoupí a soutěž se rozšíří o vítěze kvalifikačních skupin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Krajské přebory 1951/52 (listy 20*) — bez externího zdroje (DS PDF pokrývá jen kvalifikaci + Mistrovství Slovenska), k ručnímu průchodu.</t>
         </is>
       </c>
     </row>

</xml_diff>